<commit_message>
New features and updated things
</commit_message>
<xml_diff>
--- a/public/hamzamominwork.xlsx
+++ b/public/hamzamominwork.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KP-AMS\kp-ams-v2\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6A9FF1C-6904-450D-845C-D5D0C244379F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF38A44-7555-4B9A-AC79-4CA7301C7944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E3DB9CE9-8BF7-45DF-BBC9-29B65E033227}"/>
   </bookViews>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="71">
   <si>
     <t>Type of audit</t>
   </si>
@@ -243,6 +232,12 @@
   </si>
   <si>
     <t>Billed Amount</t>
+  </si>
+  <si>
+    <t>Metacast Auto Pvt Ltd</t>
+  </si>
+  <si>
+    <t>Forensic</t>
   </si>
 </sst>
 </file>
@@ -253,7 +248,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,6 +303,15 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -409,11 +413,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -489,10 +494,12 @@
     <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -824,62 +831,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{865A0D9A-F378-48EA-8985-DEBE7C20569D}">
-  <dimension ref="B2:H34"/>
+  <dimension ref="B2:J35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.26953125" style="22" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.08984375" style="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.26953125" style="22" customWidth="1"/>
+    <col min="5" max="5" width="17.08984375" style="22" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="F2" s="25">
-        <f>+SUM(F3:F34)</f>
-        <v>13465600</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="G2" s="25">
+        <f>+SUM(G3:G35)</f>
+        <v>13535400</v>
+      </c>
+      <c r="H2" s="25">
+        <f>+SUM(H3:H35)</f>
+        <v>13535400</v>
+      </c>
+      <c r="I2" s="25">
+        <f>+SUM(I3:I35)</f>
+        <v>7374600</v>
+      </c>
+      <c r="J2" s="27">
+        <f>+I2/H2</f>
+        <v>0.54483798040693299</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="17"/>
+      <c r="E3" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="H3" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="H3" s="26" t="s">
+      <c r="I3" s="26" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="18"/>
+      <c r="E4" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="F4" s="5">
-        <v>250000</v>
       </c>
       <c r="G4" s="5">
         <v>250000</v>
@@ -887,22 +906,23 @@
       <c r="H4" s="5">
         <v>250000</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I4" s="5">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="19"/>
+      <c r="E5" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="F5" s="7">
-        <v>200000</v>
       </c>
       <c r="G5" s="7">
         <v>200000</v>
@@ -910,108 +930,113 @@
       <c r="H5" s="7">
         <v>200000</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I5" s="7">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="19"/>
+      <c r="E6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="7">
+      <c r="G6" s="7">
         <v>250000</v>
       </c>
-      <c r="G6" s="7">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H6" s="7">
+        <v>250000</v>
+      </c>
+      <c r="I6" s="7"/>
+    </row>
+    <row r="7" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="19"/>
+      <c r="E7" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="7">
+      <c r="G7" s="7">
         <v>200000</v>
       </c>
-      <c r="G7" s="7">
-        <v>0</v>
-      </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H7" s="7">
+        <v>200000</v>
+      </c>
+      <c r="I7" s="7"/>
+    </row>
+    <row r="8" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="19"/>
+      <c r="E8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="F8" s="7">
-        <v>190000</v>
       </c>
       <c r="G8" s="7">
         <v>190000</v>
       </c>
       <c r="H8" s="7">
+        <v>190000</v>
+      </c>
+      <c r="I8" s="7">
         <v>100000</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="19"/>
+      <c r="E9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="7">
+      <c r="G9" s="7">
         <v>250000</v>
       </c>
-      <c r="G9" s="7">
-        <v>0</v>
-      </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H9" s="7">
+        <v>250000</v>
+      </c>
+      <c r="I9" s="7"/>
+    </row>
+    <row r="10" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="19"/>
+      <c r="E10" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="F10" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="F10" s="7">
-        <v>50000</v>
       </c>
       <c r="G10" s="7">
         <v>50000</v>
@@ -1019,502 +1044,605 @@
       <c r="H10" s="7">
         <v>50000</v>
       </c>
-    </row>
-    <row r="11" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I10" s="7">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="19"/>
+      <c r="E11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>19</v>
-      </c>
-      <c r="F11" s="7">
-        <v>2500000</v>
       </c>
       <c r="G11" s="7">
         <v>2500000</v>
       </c>
       <c r="H11" s="7">
+        <v>2500000</v>
+      </c>
+      <c r="I11" s="7">
         <v>1300000</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="19"/>
+      <c r="E12" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="F12" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="F12" s="7">
-        <v>1200000</v>
       </c>
       <c r="G12" s="7">
         <v>1200000</v>
       </c>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H12" s="7">
+        <v>1200000</v>
+      </c>
+      <c r="I12" s="7">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="19"/>
+      <c r="E13" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="7">
+      <c r="G13" s="7">
         <f>200000</f>
         <v>200000</v>
       </c>
-      <c r="G13" s="7">
+      <c r="H13" s="7">
         <v>200000</v>
       </c>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="I13" s="7">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="19"/>
+      <c r="E14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="F14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="7">
+      <c r="G14" s="7">
         <v>800000</v>
       </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H14" s="7">
+        <v>800000</v>
+      </c>
+      <c r="I14" s="7">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="19"/>
+      <c r="E15" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="F15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F15" s="7">
+      <c r="G15" s="7">
         <v>750000</v>
       </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B16" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" s="11">
-        <v>800000</v>
-      </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-    </row>
-    <row r="17" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H15" s="7">
+        <v>750000</v>
+      </c>
+      <c r="I15" s="7">
+        <v>750000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="8"/>
+      <c r="G16" s="7">
+        <v>25000</v>
+      </c>
+      <c r="H16" s="7">
+        <v>25000</v>
+      </c>
+      <c r="I16" s="7"/>
+    </row>
+    <row r="17" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B17" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="11">
-        <v>375000</v>
+      <c r="C17" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="G17" s="11">
-        <v>375000</v>
+        <v>800000</v>
       </c>
       <c r="H17" s="11">
-        <v>375000</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+        <v>800000</v>
+      </c>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B18" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="21"/>
+      <c r="E18" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="11">
+      <c r="F18" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="11">
         <v>375000</v>
       </c>
-      <c r="G18" s="11">
-        <v>0</v>
-      </c>
-      <c r="H18" s="11"/>
-    </row>
-    <row r="19" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H18" s="11">
+        <v>375000</v>
+      </c>
+      <c r="I18" s="11">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B19" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C19" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="21"/>
+      <c r="E19" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="F19" s="11">
+      <c r="F19" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="11">
         <v>375000</v>
       </c>
-      <c r="G19" s="11">
-        <v>0</v>
-      </c>
-      <c r="H19" s="11"/>
-    </row>
-    <row r="20" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H19" s="11">
+        <v>375000</v>
+      </c>
+      <c r="I19" s="11">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B20" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C20" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="21"/>
+      <c r="E20" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E20" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="F20" s="11">
+      <c r="F20" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="11">
         <v>375000</v>
       </c>
-      <c r="G20" s="11">
-        <v>0</v>
-      </c>
-      <c r="H20" s="11"/>
-    </row>
-    <row r="21" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H20" s="11">
+        <v>375000</v>
+      </c>
+      <c r="I20" s="11">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B21" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C21" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="21"/>
+      <c r="E21" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E21" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F21" s="11">
+      <c r="F21" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="11">
         <v>375000</v>
       </c>
-      <c r="G21" s="11">
-        <v>0</v>
-      </c>
-      <c r="H21" s="11"/>
-    </row>
-    <row r="22" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H21" s="11">
+        <v>375000</v>
+      </c>
+      <c r="I21" s="11">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B22" s="9" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C22" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="21"/>
+      <c r="E22" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="F22" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G22" s="11">
+        <v>375000</v>
+      </c>
+      <c r="H22" s="11">
+        <v>375000</v>
+      </c>
+      <c r="I22" s="11">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B23" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="F22" s="14">
-        <v>1500000</v>
-      </c>
-      <c r="G22" s="14">
-        <v>150000</v>
-      </c>
-      <c r="H22" s="14">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B23" s="9" t="s">
-        <v>63</v>
       </c>
       <c r="C23" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="21"/>
+      <c r="E23" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="F23" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="14">
+        <v>1500000</v>
+      </c>
+      <c r="H23" s="14">
+        <v>1500000</v>
+      </c>
+      <c r="I23" s="14">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B24" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="14">
+      <c r="G24" s="14">
         <f>125000*2</f>
         <v>250000</v>
       </c>
-      <c r="G23" s="14">
+      <c r="H24" s="14">
         <v>250000</v>
       </c>
-      <c r="H23" s="14">
+      <c r="I24" s="14">
         <v>250000</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B24" s="9" t="s">
+    <row r="25" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B25" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C25" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="D25" s="21"/>
+      <c r="E25" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="F25" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="14">
+      <c r="G25" s="14">
         <v>300000</v>
       </c>
-      <c r="G24" s="14">
+      <c r="H25" s="14">
+        <v>300000</v>
+      </c>
+      <c r="I25" s="14">
         <v>200000</v>
       </c>
-      <c r="H24" s="14">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B25" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D25" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="16">
-        <v>145600</v>
-      </c>
-      <c r="G25" s="16">
-        <v>49600</v>
-      </c>
-      <c r="H25" s="16">
-        <v>49600</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B26" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F26" s="16">
-        <v>450000</v>
+      <c r="C26" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="20"/>
+      <c r="E26" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>41</v>
       </c>
       <c r="G26" s="16">
-        <v>0</v>
-      </c>
-      <c r="H26" s="16"/>
-    </row>
-    <row r="27" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+        <v>190400</v>
+      </c>
+      <c r="H26" s="16">
+        <v>190400</v>
+      </c>
+      <c r="I26" s="16">
+        <v>49600</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B27" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C27" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="E27" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="F27" s="16">
-        <v>425000</v>
-      </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-    </row>
-    <row r="28" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F27" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="16">
+        <v>450000</v>
+      </c>
+      <c r="H27" s="16">
+        <v>450000</v>
+      </c>
+      <c r="I27" s="16"/>
+    </row>
+    <row r="28" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B28" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C28" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="F28" s="16">
-        <v>250000</v>
-      </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-    </row>
-    <row r="29" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F28" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G28" s="16">
+        <v>425000</v>
+      </c>
+      <c r="H28" s="16">
+        <v>425000</v>
+      </c>
+      <c r="I28" s="16"/>
+    </row>
+    <row r="29" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B29" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C29" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F29" s="16">
+      <c r="F29" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G29" s="16">
         <v>250000</v>
       </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-    </row>
-    <row r="30" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H29" s="16">
+        <v>250000</v>
+      </c>
+      <c r="I29" s="16"/>
+    </row>
+    <row r="30" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B30" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E30" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="F30" s="16">
-        <v>150000</v>
-      </c>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F30" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30" s="16">
+        <v>250000</v>
+      </c>
+      <c r="H30" s="16">
+        <v>250000</v>
+      </c>
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B31" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="F31" s="16">
-        <v>50000</v>
-      </c>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-    </row>
-    <row r="32" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F31" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G31" s="16">
+        <v>150000</v>
+      </c>
+      <c r="H31" s="16">
+        <v>150000</v>
+      </c>
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B32" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C32" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="D32" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E32" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="F32" s="16">
+      <c r="F32" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G32" s="16">
         <v>50000</v>
       </c>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H32" s="16">
+        <v>50000</v>
+      </c>
+      <c r="I32" s="16"/>
+    </row>
+    <row r="33" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B33" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C33" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D33" s="21" t="s">
+      <c r="D33" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E33" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="F33" s="16">
-        <v>80000</v>
-      </c>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-    </row>
-    <row r="34" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F33" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G33" s="16">
+        <v>50000</v>
+      </c>
+      <c r="H33" s="16">
+        <v>50000</v>
+      </c>
+      <c r="I33" s="16"/>
+    </row>
+    <row r="34" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B34" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C34" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="F34" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" s="16">
+        <v>80000</v>
+      </c>
+      <c r="H34" s="16">
+        <v>80000</v>
+      </c>
+      <c r="I34" s="16"/>
+    </row>
+    <row r="35" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B35" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D35" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F34" s="16">
+      <c r="E35" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G35" s="16">
         <v>50000</v>
       </c>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
+      <c r="H35" s="16">
+        <v>50000</v>
+      </c>
+      <c r="I35" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated all of the things also bug fixes
</commit_message>
<xml_diff>
--- a/public/hamzamominwork.xlsx
+++ b/public/hamzamominwork.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KP-AMS\kp-ams-v2\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB513B37-BDC3-4A4B-A26A-52511A276A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3743C2-1E49-459C-8F2C-D03238B00F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E3DB9CE9-8BF7-45DF-BBC9-29B65E033227}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="70">
   <si>
     <t>Type of audit</t>
   </si>
@@ -220,9 +220,6 @@
   </si>
   <si>
     <t>John Deere India Pvt Ltd</t>
-  </si>
-  <si>
-    <t>Mahindra and Mahindra Lt</t>
   </si>
   <si>
     <t>Assignment Specs</t>
@@ -871,7 +868,7 @@
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>2</v>
@@ -880,10 +877,10 @@
         <v>3</v>
       </c>
       <c r="H3" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I3" s="26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
@@ -1174,11 +1171,11 @@
         <v>52</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D16" s="19"/>
       <c r="E16" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="7">
@@ -1432,12 +1429,10 @@
       <c r="B27" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="15" t="s">
+      <c r="C27" s="15" t="s">
         <v>43</v>
       </c>
+      <c r="D27" s="15"/>
       <c r="E27" s="21" t="s">
         <v>42</v>
       </c>
@@ -1456,12 +1451,10 @@
       <c r="B28" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D28" s="15" t="s">
+      <c r="C28" s="15" t="s">
         <v>44</v>
       </c>
+      <c r="D28" s="15"/>
       <c r="E28" s="21" t="s">
         <v>42</v>
       </c>
@@ -1480,12 +1473,10 @@
       <c r="B29" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="15" t="s">
+      <c r="C29" s="15" t="s">
         <v>45</v>
       </c>
+      <c r="D29" s="15"/>
       <c r="E29" s="21" t="s">
         <v>42</v>
       </c>
@@ -1504,12 +1495,10 @@
       <c r="B30" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" s="15" t="s">
+      <c r="C30" s="15" t="s">
         <v>46</v>
       </c>
+      <c r="D30" s="15"/>
       <c r="E30" s="21" t="s">
         <v>42</v>
       </c>
@@ -1528,12 +1517,10 @@
       <c r="B31" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="15" t="s">
         <v>47</v>
       </c>
+      <c r="D31" s="15"/>
       <c r="E31" s="21" t="s">
         <v>42</v>
       </c>
@@ -1552,12 +1539,10 @@
       <c r="B32" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="15" t="s">
+      <c r="C32" s="15" t="s">
         <v>48</v>
       </c>
+      <c r="D32" s="15"/>
       <c r="E32" s="21" t="s">
         <v>42</v>
       </c>
@@ -1576,12 +1561,10 @@
       <c r="B33" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" s="15" t="s">
+      <c r="C33" s="15" t="s">
         <v>49</v>
       </c>
+      <c r="D33" s="15"/>
       <c r="E33" s="21" t="s">
         <v>42</v>
       </c>
@@ -1600,12 +1583,10 @@
       <c r="B34" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D34" s="15" t="s">
+      <c r="C34" s="15" t="s">
         <v>50</v>
       </c>
+      <c r="D34" s="15"/>
       <c r="E34" s="21" t="s">
         <v>42</v>
       </c>
@@ -1624,12 +1605,10 @@
       <c r="B35" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" s="15" t="s">
+      <c r="C35" s="15" t="s">
         <v>51</v>
       </c>
+      <c r="D35" s="15"/>
       <c r="E35" s="21" t="s">
         <v>42</v>
       </c>

</xml_diff>